<commit_message>
Simplify dashboard to requested layout with color-coded groups and charts
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Zs2f4qGzAhq6ccis9Pnwf
</commit_message>
<xml_diff>
--- a/Data_Analysis_Dashboard.xlsx
+++ b/Data_Analysis_Dashboard.xlsx
@@ -20,54 +20,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="19">
   <si>
-    <t xml:space="preserve">لوحة تحليل البيانات | Data Analysis Dashboard</t>
+    <t xml:space="preserve">لوحة تحليل نتائج الطلاب</t>
   </si>
   <si>
-    <t xml:space="preserve">اسم المعلم | Teacher</t>
+    <t xml:space="preserve">اسم المعلم</t>
   </si>
   <si>
-    <t xml:space="preserve">Mr. Example</t>
+    <t xml:space="preserve">اكتب الاسم هنا</t>
   </si>
   <si>
-    <t xml:space="preserve">الصف | Class</t>
+    <t xml:space="preserve">الصف</t>
   </si>
   <si>
-    <t xml:space="preserve">Grade 10A</t>
+    <t xml:space="preserve">10A</t>
   </si>
   <si>
-    <t xml:space="preserve">عدد الطلاب | Students</t>
+    <t xml:space="preserve">عدد الطلاب</t>
   </si>
   <si>
-    <t xml:space="preserve">الخلايا الصفراء (خط أزرق) = إدخال | عدّل الأرقام المثال بأرقامك</t>
-  </si>
-  <si>
-    <t xml:space="preserve">سلّم التقدير (حسب نسبة At+Above) | Rating scale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">من (≥)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Outstanding | متميز</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Very Good | جيد جدًا</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Good | جيد</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acceptable | مقبول</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weak | ضعيف</t>
-  </si>
-  <si>
-    <t xml:space="preserve">الحدود افتراضية قابلة للتعديل (ليست رسمية)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">الصف كاملًا | Whole Class</t>
+    <t xml:space="preserve">الصف كاملًا</t>
   </si>
   <si>
     <t xml:space="preserve">At + Above</t>
@@ -76,28 +49,34 @@
     <t xml:space="preserve">Above</t>
   </si>
   <si>
-    <t xml:space="preserve">التقدير | Rating</t>
+    <t xml:space="preserve">التقدير  Rating</t>
   </si>
   <si>
-    <t xml:space="preserve">التحصيل | Attainment (عدد)</t>
+    <t xml:space="preserve">التحصيل  Attainment</t>
   </si>
   <si>
-    <t xml:space="preserve">التحصيل | Attainment (%)</t>
+    <t xml:space="preserve">Good</t>
   </si>
   <si>
-    <t xml:space="preserve">التقدم | Progress (عدد)</t>
+    <t xml:space="preserve">التقدم  Progress</t>
   </si>
   <si>
-    <t xml:space="preserve">التقدم | Progress (%)</t>
+    <t xml:space="preserve">الإماراتيون</t>
   </si>
   <si>
-    <t xml:space="preserve">الإماراتيون | Emiratis</t>
+    <t xml:space="preserve">Acceptable</t>
   </si>
   <si>
-    <t xml:space="preserve">السندو | SEND</t>
+    <t xml:space="preserve">السندو  SEND</t>
   </si>
   <si>
-    <t xml:space="preserve">الجيفتد والتالنتد | Gifted &amp; Talented</t>
+    <t xml:space="preserve">الجيفتد والتالنتد  G&amp;T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outstanding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very Good</t>
   </si>
 </sst>
 </file>
@@ -106,10 +85,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0%"/>
-    <numFmt numFmtId="166" formatCode="&quot;عدد: &quot;0"/>
+    <numFmt numFmtId="165" formatCode="&quot;الطلاب: &quot;0"/>
+    <numFmt numFmtId="166" formatCode="0%"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -134,39 +113,8 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="16"/>
+      <sz val="18"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="9"/>
-      <color rgb="FF666666"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -181,8 +129,48 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="11"/>
+      <sz val="13"/>
+      <color rgb="FF1F3864"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="15"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="14"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FFFFFF99"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -195,20 +183,20 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -223,36 +211,66 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF9C4"/>
-        <bgColor rgb="FFFFFF99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF7F7F7F"/>
-        <bgColor rgb="FF878787"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF2E75B6"/>
         <bgColor rgb="FF0066CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFDDEBF7"/>
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDDEBF7"/>
-        <bgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FF8FAADC"/>
+        <bgColor rgb="FF969696"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF548235"/>
+        <bgColor rgb="FF878787"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA9D18E"/>
+        <bgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC55A11"/>
+        <bgColor rgb="FFFF5050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4B183"/>
+        <bgColor rgb="FFFFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor rgb="FF993366"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9A3E0"/>
+        <bgColor rgb="FFBFBFBF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -262,29 +280,89 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FF999999"/>
+        <color rgb="FFBFBFBF"/>
       </left>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
+      <right/>
       <top style="thin">
-        <color rgb="FF999999"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF999999"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FF999999"/>
+        <color rgb="FFBFBFBF"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
       <top style="thin">
-        <color rgb="FF999999"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF999999"/>
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F3864"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium">
+        <color rgb="FF548235"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF548235"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF548235"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF548235"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium">
+        <color rgb="FFC55A11"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC55A11"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC55A11"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC55A11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium">
+        <color rgb="FF7030A0"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF7030A0"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF7030A0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF7030A0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -314,64 +392,116 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="6" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -384,6 +514,78 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFD966"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4B183"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -397,14 +599,14 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF548235"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF7F7F7F"/>
+      <rgbColor rgb="FFBFBFBF"/>
       <rgbColor rgb="FF878787"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF9C4"/>
+      <rgbColor rgb="FF8FAADC"/>
+      <rgbColor rgb="FF7030A0"/>
+      <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFDDEBF7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -419,26 +621,26 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFF2F2F2"/>
+      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFA9D18E"/>
+      <rgbColor rgb="FFF4B183"/>
+      <rgbColor rgb="FFC9A3E0"/>
+      <rgbColor rgb="FFFFD966"/>
       <rgbColor rgb="FF2E75B6"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FF92D050"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFED7D31"/>
-      <rgbColor rgb="FF666666"/>
-      <rgbColor rgb="FF999999"/>
+      <rgbColor rgb="FFFF5050"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF1F3864"/>
-      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF00B050"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFC55A11"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
@@ -473,7 +675,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>الصف كاملًا | Whole Class</a:t>
+              <a:t>الصف كاملًا</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -497,21 +699,23 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التحصيل Attainment"</c:f>
+              <c:f>"التحصيل"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التحصيل Attainment</c:v>
+                  <c:v>التحصيل</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="2e75b6"/>
+              <a:srgbClr val="1f3864"/>
             </a:solidFill>
             <a:ln w="0">
-              <a:noFill/>
+              <a:solidFill>
+                <a:srgbClr val="1f3864"/>
+              </a:solidFill>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
@@ -531,10 +735,10 @@
               </a:p>
             </c:txPr>
             <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="1"/>
+            <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
@@ -546,7 +750,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$17:$D$17</c:f>
+              <c:f>Dashboard!$C$7:$D$7</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -564,15 +768,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$19:$D$19</c:f>
+              <c:f>Dashboard!$C$8:$D$8</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.714285714285714</c:v>
+                  <c:v>0.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.285714285714286</c:v>
+                  <c:v>0.35</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -583,21 +787,23 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التقدم Progress"</c:f>
+              <c:f>"التقدم"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التقدم Progress</c:v>
+                  <c:v>التقدم</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="ed7d31"/>
+              <a:srgbClr val="8faadc"/>
             </a:solidFill>
             <a:ln w="0">
-              <a:noFill/>
+              <a:solidFill>
+                <a:srgbClr val="8faadc"/>
+              </a:solidFill>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
@@ -617,10 +823,10 @@
               </a:p>
             </c:txPr>
             <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="1"/>
+            <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
@@ -632,7 +838,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$17:$D$17</c:f>
+              <c:f>Dashboard!$C$7:$D$7</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -650,27 +856,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$22:$D$22</c:f>
+              <c:f>Dashboard!$C$9:$D$9</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.642857142857143</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.25</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:gapWidth val="150"/>
+        <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="6901770"/>
-        <c:axId val="94392475"/>
+        <c:axId val="81562439"/>
+        <c:axId val="27731922"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="6901770"/>
+        <c:axId val="81562439"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -702,7 +908,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94392475"/>
+        <c:crossAx val="27731922"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -710,7 +916,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94392475"/>
+        <c:axId val="27731922"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -718,16 +924,6 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="878787"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
         <c:numFmt formatCode="0%" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -754,7 +950,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6901770"/>
+        <c:crossAx val="81562439"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -832,7 +1028,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>الإماراتيون | Emiratis</a:t>
+              <a:t>الإماراتيون</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -856,21 +1052,23 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التحصيل Attainment"</c:f>
+              <c:f>"التحصيل"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التحصيل Attainment</c:v>
+                  <c:v>التحصيل</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="2e75b6"/>
+              <a:srgbClr val="548235"/>
             </a:solidFill>
             <a:ln w="0">
-              <a:noFill/>
+              <a:solidFill>
+                <a:srgbClr val="548235"/>
+              </a:solidFill>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
@@ -890,10 +1088,10 @@
               </a:p>
             </c:txPr>
             <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="1"/>
+            <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
@@ -905,7 +1103,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$30:$D$30</c:f>
+              <c:f>Dashboard!$C$15:$D$15</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -923,15 +1121,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$32:$D$32</c:f>
+              <c:f>Dashboard!$C$16:$D$16</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.875</c:v>
+                  <c:v>0.7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.5</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -942,21 +1140,23 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التقدم Progress"</c:f>
+              <c:f>"التقدم"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التقدم Progress</c:v>
+                  <c:v>التقدم</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="ed7d31"/>
+              <a:srgbClr val="a9d18e"/>
             </a:solidFill>
             <a:ln w="0">
-              <a:noFill/>
+              <a:solidFill>
+                <a:srgbClr val="a9d18e"/>
+              </a:solidFill>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
@@ -976,10 +1176,10 @@
               </a:p>
             </c:txPr>
             <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="1"/>
+            <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
@@ -991,7 +1191,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$30:$D$30</c:f>
+              <c:f>Dashboard!$C$15:$D$15</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -1009,27 +1209,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$35:$D$35</c:f>
+              <c:f>Dashboard!$C$17:$D$17</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.75</c:v>
+                  <c:v>0.65</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.375</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:gapWidth val="150"/>
+        <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="74811583"/>
-        <c:axId val="11967405"/>
+        <c:axId val="5298332"/>
+        <c:axId val="12279837"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="74811583"/>
+        <c:axId val="5298332"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1061,7 +1261,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11967405"/>
+        <c:crossAx val="12279837"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1069,7 +1269,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11967405"/>
+        <c:axId val="12279837"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1077,16 +1277,6 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="878787"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
         <c:numFmt formatCode="0%" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1113,7 +1303,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74811583"/>
+        <c:crossAx val="5298332"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1191,7 +1381,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>السندو | SEND</a:t>
+              <a:t>السندو  SEND</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1215,21 +1405,23 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التحصيل Attainment"</c:f>
+              <c:f>"التحصيل"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التحصيل Attainment</c:v>
+                  <c:v>التحصيل</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="2e75b6"/>
+              <a:srgbClr val="c55a11"/>
             </a:solidFill>
             <a:ln w="0">
-              <a:noFill/>
+              <a:solidFill>
+                <a:srgbClr val="c55a11"/>
+              </a:solidFill>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
@@ -1249,10 +1441,10 @@
               </a:p>
             </c:txPr>
             <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="1"/>
+            <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
@@ -1264,7 +1456,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$43:$D$43</c:f>
+              <c:f>Dashboard!$C$23:$D$23</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -1282,15 +1474,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$45:$D$45</c:f>
+              <c:f>Dashboard!$C$24:$D$24</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.75</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.25</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1301,21 +1493,23 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التقدم Progress"</c:f>
+              <c:f>"التقدم"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التقدم Progress</c:v>
+                  <c:v>التقدم</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="ed7d31"/>
+              <a:srgbClr val="f4b183"/>
             </a:solidFill>
             <a:ln w="0">
-              <a:noFill/>
+              <a:solidFill>
+                <a:srgbClr val="f4b183"/>
+              </a:solidFill>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
@@ -1335,10 +1529,10 @@
               </a:p>
             </c:txPr>
             <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="1"/>
+            <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
@@ -1350,7 +1544,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$43:$D$43</c:f>
+              <c:f>Dashboard!$C$23:$D$23</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -1368,27 +1562,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$48:$D$48</c:f>
+              <c:f>Dashboard!$C$25:$D$25</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.5</c:v>
+                  <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:gapWidth val="150"/>
+        <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="98779583"/>
-        <c:axId val="22747865"/>
+        <c:axId val="61430187"/>
+        <c:axId val="43799199"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="98779583"/>
+        <c:axId val="61430187"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1420,7 +1614,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22747865"/>
+        <c:crossAx val="43799199"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1428,7 +1622,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22747865"/>
+        <c:axId val="43799199"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1436,16 +1630,6 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="878787"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
         <c:numFmt formatCode="0%" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1472,7 +1656,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98779583"/>
+        <c:crossAx val="61430187"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1550,7 +1734,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>الجيفتد والتالنتد | Gifted &amp; Talented</a:t>
+              <a:t>الجيفتد والتالنتد  G&amp;T</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1574,21 +1758,23 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التحصيل Attainment"</c:f>
+              <c:f>"التحصيل"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التحصيل Attainment</c:v>
+                  <c:v>التحصيل</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="2e75b6"/>
+              <a:srgbClr val="7030a0"/>
             </a:solidFill>
             <a:ln w="0">
-              <a:noFill/>
+              <a:solidFill>
+                <a:srgbClr val="7030a0"/>
+              </a:solidFill>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
@@ -1608,10 +1794,10 @@
               </a:p>
             </c:txPr>
             <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="1"/>
+            <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
@@ -1623,7 +1809,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$56:$D$56</c:f>
+              <c:f>Dashboard!$C$31:$D$31</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -1641,15 +1827,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$58:$D$58</c:f>
+              <c:f>Dashboard!$C$32:$D$32</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.666666666666667</c:v>
+                  <c:v>0.6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1660,21 +1846,23 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التقدم Progress"</c:f>
+              <c:f>"التقدم"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التقدم Progress</c:v>
+                  <c:v>التقدم</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="ed7d31"/>
+              <a:srgbClr val="c9a3e0"/>
             </a:solidFill>
             <a:ln w="0">
-              <a:noFill/>
+              <a:solidFill>
+                <a:srgbClr val="c9a3e0"/>
+              </a:solidFill>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
@@ -1694,10 +1882,10 @@
               </a:p>
             </c:txPr>
             <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="1"/>
+            <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
@@ -1709,7 +1897,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$56:$D$56</c:f>
+              <c:f>Dashboard!$C$31:$D$31</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -1727,27 +1915,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$61:$D$61</c:f>
+              <c:f>Dashboard!$C$33:$D$33</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
+                  <c:v>0.85</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.666666666666667</c:v>
+                  <c:v>0.55</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:gapWidth val="150"/>
+        <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="74579526"/>
-        <c:axId val="9362545"/>
+        <c:axId val="75508505"/>
+        <c:axId val="82428111"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="74579526"/>
+        <c:axId val="75508505"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1779,7 +1967,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9362545"/>
+        <c:crossAx val="82428111"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1787,7 +1975,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9362545"/>
+        <c:axId val="82428111"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1795,16 +1983,6 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="878787"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
         <c:numFmt formatCode="0%" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1831,7 +2009,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74579526"/>
+        <c:crossAx val="75508505"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1888,15 +2066,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>-79200</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:colOff>-39240</xdr:colOff>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>50400</xdr:rowOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>156960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1904,8 +2082,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-9668880" y="3048120"/>
-        <a:ext cx="3959640" cy="2231640"/>
+        <a:off x="-10170000" y="1562040"/>
+        <a:ext cx="4319640" cy="1871640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1918,15 +2096,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>-79200</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:colOff>-39240</xdr:colOff>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>130320</xdr:rowOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>156960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1934,8 +2112,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-9668880" y="5610240"/>
-        <a:ext cx="3959640" cy="2231640"/>
+        <a:off x="-10170000" y="3657600"/>
+        <a:ext cx="4319640" cy="1871640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1948,15 +2126,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>-79200</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>79920</xdr:rowOff>
+      <xdr:colOff>-39240</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>170280</xdr:rowOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>157320</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1964,8 +2142,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-9668880" y="8172360"/>
-        <a:ext cx="3959640" cy="2231640"/>
+        <a:off x="-10170000" y="5753160"/>
+        <a:ext cx="4319640" cy="1871640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1978,15 +2156,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>-79200</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>120240</xdr:rowOff>
+      <xdr:colOff>-39240</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>60120</xdr:rowOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>157320</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1994,8 +2172,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-9668880" y="10734840"/>
-        <a:ext cx="3959640" cy="2231640"/>
+        <a:off x="-10170000" y="7848720"/>
+        <a:ext cx="4319640" cy="1871640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2188,17 +2366,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E61"/>
+  <dimension ref="B1:E33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="3"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2206,7 +2384,7 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2216,7 +2394,7 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
@@ -2226,7 +2404,7 @@
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
@@ -2236,431 +2414,248 @@
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="6"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="6"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="6"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E13" s="6"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="9" t="n">
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="5" t="n">
         <f aca="false">C4</f>
         <v>28</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="10"/>
-      <c r="C17" s="10" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="6"/>
+      <c r="C7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="11" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="12"/>
+      <c r="C15" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="18"/>
+      <c r="C23" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D24" s="20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E24" s="21" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="20" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D25" s="20" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E25" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="E18" s="11"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="13" t="n">
-        <f aca="false">IF($E$16&gt;0,C18/$E$16,0)</f>
-        <v>0.714285714285714</v>
-      </c>
-      <c r="D19" s="13" t="n">
-        <f aca="false">IF($E$16&gt;0,D18/$E$16,0)</f>
-        <v>0.285714285714286</v>
-      </c>
-      <c r="E19" s="12" t="str">
-        <f aca="false">INDEX($D$9:$D$13,MATCH(TRUE(),INDEX(C19&gt;=$C$9:$C$13,0),0))</f>
-        <v>Good | جيد</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="E21" s="11"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" s="13" t="n">
-        <f aca="false">IF($E$16&gt;0,C21/$E$16,0)</f>
-        <v>0.642857142857143</v>
-      </c>
-      <c r="D22" s="13" t="n">
-        <f aca="false">IF($E$16&gt;0,D21/$E$16,0)</f>
-        <v>0.25</v>
-      </c>
-      <c r="E22" s="12" t="str">
-        <f aca="false">INDEX($D$9:$D$13,MATCH(TRUE(),INDEX(C22&gt;=$C$9:$C$13,0),0))</f>
-        <v>Good | جيد</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="14" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="10"/>
-      <c r="C30" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>18</v>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="23" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C31" s="3" t="n">
+      <c r="B31" s="24"/>
+      <c r="C31" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E31" s="11"/>
+      <c r="D31" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31" s="24" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C32" s="13" t="n">
-        <f aca="false">IF($E$29&gt;0,C31/$E$29,0)</f>
-        <v>0.875</v>
-      </c>
-      <c r="D32" s="13" t="n">
-        <f aca="false">IF($E$29&gt;0,D31/$E$29,0)</f>
-        <v>0.5</v>
-      </c>
-      <c r="E32" s="12" t="str">
-        <f aca="false">INDEX($D$9:$D$13,MATCH(TRUE(),INDEX(C32&gt;=$C$9:$C$13,0),0))</f>
-        <v>Very Good | جيد جدًا</v>
+    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="26" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D32" s="26" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E32" s="27" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C34" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E34" s="11"/>
-    </row>
-    <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="C35" s="13" t="n">
-        <f aca="false">IF($E$29&gt;0,C34/$E$29,0)</f>
-        <v>0.75</v>
-      </c>
-      <c r="D35" s="13" t="n">
-        <f aca="false">IF($E$29&gt;0,D34/$E$29,0)</f>
-        <v>0.375</v>
-      </c>
-      <c r="E35" s="12" t="str">
-        <f aca="false">INDEX($D$9:$D$13,MATCH(TRUE(),INDEX(C35&gt;=$C$9:$C$13,0),0))</f>
-        <v>Very Good | جيد جدًا</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
-      <c r="E42" s="14" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="10"/>
-      <c r="C43" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E43" s="10" t="s">
+    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" s="26" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D33" s="26" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E33" s="27" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C44" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D44" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" s="11"/>
-    </row>
-    <row r="45" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C45" s="13" t="n">
-        <f aca="false">IF($E$42&gt;0,C44/$E$42,0)</f>
-        <v>0.75</v>
-      </c>
-      <c r="D45" s="13" t="n">
-        <f aca="false">IF($E$42&gt;0,D44/$E$42,0)</f>
-        <v>0.25</v>
-      </c>
-      <c r="E45" s="12" t="str">
-        <f aca="false">INDEX($D$9:$D$13,MATCH(TRUE(),INDEX(C45&gt;=$C$9:$C$13,0),0))</f>
-        <v>Very Good | جيد جدًا</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C47" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D47" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E47" s="11"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="C48" s="13" t="n">
-        <f aca="false">IF($E$42&gt;0,C47/$E$42,0)</f>
-        <v>0.5</v>
-      </c>
-      <c r="D48" s="13" t="n">
-        <f aca="false">IF($E$42&gt;0,D47/$E$42,0)</f>
-        <v>0</v>
-      </c>
-      <c r="E48" s="12" t="str">
-        <f aca="false">INDEX($D$9:$D$13,MATCH(TRUE(),INDEX(C48&gt;=$C$9:$C$13,0),0))</f>
-        <v>Acceptable | مقبول</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B55" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C55" s="8"/>
-      <c r="D55" s="8"/>
-      <c r="E55" s="14" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="10"/>
-      <c r="C56" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D56" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E56" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C57" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D57" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E57" s="11"/>
-    </row>
-    <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C58" s="13" t="n">
-        <f aca="false">IF($E$55&gt;0,C57/$E$55,0)</f>
-        <v>1</v>
-      </c>
-      <c r="D58" s="13" t="n">
-        <f aca="false">IF($E$55&gt;0,D57/$E$55,0)</f>
-        <v>0.666666666666667</v>
-      </c>
-      <c r="E58" s="12" t="str">
-        <f aca="false">INDEX($D$9:$D$13,MATCH(TRUE(),INDEX(C58&gt;=$C$9:$C$13,0),0))</f>
-        <v>Outstanding | متميز</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C60" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D60" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E60" s="11"/>
-    </row>
-    <row r="61" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="C61" s="13" t="n">
-        <f aca="false">IF($E$55&gt;0,C60/$E$55,0)</f>
-        <v>1</v>
-      </c>
-      <c r="D61" s="13" t="n">
-        <f aca="false">IF($E$55&gt;0,D60/$E$55,0)</f>
-        <v>0.666666666666667</v>
-      </c>
-      <c r="E61" s="12" t="str">
-        <f aca="false">INDEX($D$9:$D$13,MATCH(TRUE(),INDEX(C61&gt;=$C$9:$C$13,0),0))</f>
-        <v>Outstanding | متميز</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="8">
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C4:E4"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B30:D30"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation allowBlank="false" error="أدخل رقمًا صحيحًا" errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C18:D18 C21:D21 C31:D31 C34:D34 C44:D44 C47:D47 C57:D57 C60:D60" type="whole">
+  <conditionalFormatting sqref="E8:E40">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>E8="Outstanding"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>E8="Very Good"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>E8="Good"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>E8="Acceptable"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+      <formula>E8="Weak"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E8:E9 E16:E17 E24:E25 E32:E33" type="list">
+      <formula1>"Outstanding,Very Good,Good,Acceptable,Weak"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="أدخل نسبة بين 0% و100%" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C8:D9 C16:D17 C24:D25 C32:D33" type="decimal">
       <formula1>0</formula1>
-      <formula2>0</formula2>
+      <formula2>1</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
Redesign dashboard: 2x2 group boxes with charts section below
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Zs2f4qGzAhq6ccis9Pnwf
</commit_message>
<xml_diff>
--- a/Data_Analysis_Dashboard.xlsx
+++ b/Data_Analysis_Dashboard.xlsx
@@ -10,6 +10,9 @@
   <sheets>
     <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Dashboard!$A$1:$K$50</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -20,27 +23,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="20">
   <si>
-    <t xml:space="preserve">لوحة تحليل نتائج الطلاب</t>
+    <t xml:space="preserve">لوحة تحليل التحصيل والتقدم  |  Attainment &amp; Progress Dashboard</t>
   </si>
   <si>
-    <t xml:space="preserve">اسم المعلم</t>
+    <t xml:space="preserve">عدد الطلاب  Students</t>
   </si>
   <si>
-    <t xml:space="preserve">اكتب الاسم هنا</t>
+    <t xml:space="preserve">الصف  Class</t>
   </si>
   <si>
-    <t xml:space="preserve">الصف</t>
+    <t xml:space="preserve">اسم المعلم  Teacher</t>
   </si>
   <si>
     <t xml:space="preserve">10A</t>
   </si>
   <si>
-    <t xml:space="preserve">عدد الطلاب</t>
+    <t xml:space="preserve">اكتب اسم المعلم</t>
   </si>
   <si>
-    <t xml:space="preserve">الصف كاملًا</t>
+    <t xml:space="preserve">الإماراتيون  Emiratis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الصف كاملًا  Whole Class</t>
   </si>
   <si>
     <t xml:space="preserve">At + Above</t>
@@ -61,22 +67,22 @@
     <t xml:space="preserve">التقدم  Progress</t>
   </si>
   <si>
-    <t xml:space="preserve">الإماراتيون</t>
-  </si>
-  <si>
     <t xml:space="preserve">Acceptable</t>
   </si>
   <si>
-    <t xml:space="preserve">السندو  SEND</t>
+    <t xml:space="preserve">الجيفتد والتالنتد  G&amp;T</t>
   </si>
   <si>
-    <t xml:space="preserve">الجيفتد والتالنتد  G&amp;T</t>
+    <t xml:space="preserve">السندو  SEND</t>
   </si>
   <si>
     <t xml:space="preserve">Outstanding</t>
   </si>
   <si>
     <t xml:space="preserve">Very Good</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الرسوم البيانية  |  Charts</t>
   </si>
 </sst>
 </file>
@@ -88,7 +94,7 @@
     <numFmt numFmtId="165" formatCode="&quot;الطلاب: &quot;0"/>
     <numFmt numFmtId="166" formatCode="0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -121,6 +127,38 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="14"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FFFFE699"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
@@ -129,8 +167,8 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="13"/>
-      <color rgb="FF1F3864"/>
+      <sz val="11"/>
+      <color rgb="FF1A1A1A"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -138,22 +176,6 @@
     <font>
       <b val="true"/>
       <sz val="15"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="14"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -169,8 +191,8 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="12"/>
-      <color rgb="FFFFFF99"/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -183,14 +205,14 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
+      <b val="true"/>
+      <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="18"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -205,72 +227,72 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
-        <bgColor rgb="FF333333"/>
+        <fgColor rgb="FFF3F5F9"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2E75B6"/>
-        <bgColor rgb="FF0066CC"/>
+        <fgColor rgb="FF14213D"/>
+        <bgColor rgb="FF1A1A1A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDDEBF7"/>
-        <bgColor rgb="FFD9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF8FAADC"/>
-        <bgColor rgb="FF969696"/>
+        <fgColor rgb="FF3D5A80"/>
+        <bgColor rgb="FF4F6D9A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFF3F5F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF548235"/>
-        <bgColor rgb="FF878787"/>
+        <fgColor rgb="FF0B7A75"/>
+        <bgColor rgb="FF008080"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA9D18E"/>
-        <bgColor rgb="FF92D050"/>
+        <fgColor rgb="FF7FC8C3"/>
+        <bgColor rgb="FFC0C0C0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC55A11"/>
-        <bgColor rgb="FFFF5050"/>
+        <fgColor rgb="FF4F6D9A"/>
+        <bgColor rgb="FF3D5A80"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF4B183"/>
-        <bgColor rgb="FFFFD966"/>
+        <fgColor rgb="FF8E2C7D"/>
+        <bgColor rgb="FF800080"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF7030A0"/>
-        <bgColor rgb="FF993366"/>
+        <fgColor rgb="FFD1621B"/>
+        <bgColor rgb="FFE63946"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC9A3E0"/>
-        <bgColor rgb="FFBFBFBF"/>
+        <fgColor rgb="FFD3A0C8"/>
+        <bgColor rgb="FFFF99CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2B27F"/>
+        <bgColor rgb="FFF4A261"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -280,89 +302,76 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFBFBFBF"/>
+        <color rgb="FFD9D9D9"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
       <top style="thin">
-        <color rgb="FFBFBFBF"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFBFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin">
-        <color rgb="FFBFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFBFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFBFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFBFBFBF"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="medium">
-        <color rgb="FF1F3864"/>
+        <color rgb="FF0B7A75"/>
       </left>
       <right style="medium">
-        <color rgb="FF1F3864"/>
+        <color rgb="FF0B7A75"/>
       </right>
       <top style="medium">
-        <color rgb="FF1F3864"/>
+        <color rgb="FF0B7A75"/>
       </top>
       <bottom style="medium">
-        <color rgb="FF1F3864"/>
+        <color rgb="FF0B7A75"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="medium">
-        <color rgb="FF548235"/>
+        <color rgb="FF14213D"/>
       </left>
       <right style="medium">
-        <color rgb="FF548235"/>
+        <color rgb="FF14213D"/>
       </right>
       <top style="medium">
-        <color rgb="FF548235"/>
+        <color rgb="FF14213D"/>
       </top>
       <bottom style="medium">
-        <color rgb="FF548235"/>
+        <color rgb="FF14213D"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="medium">
-        <color rgb="FFC55A11"/>
+        <color rgb="FF8E2C7D"/>
       </left>
       <right style="medium">
-        <color rgb="FFC55A11"/>
+        <color rgb="FF8E2C7D"/>
       </right>
       <top style="medium">
-        <color rgb="FFC55A11"/>
+        <color rgb="FF8E2C7D"/>
       </top>
       <bottom style="medium">
-        <color rgb="FFC55A11"/>
+        <color rgb="FF8E2C7D"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="medium">
-        <color rgb="FF7030A0"/>
+        <color rgb="FFD1621B"/>
       </left>
       <right style="medium">
-        <color rgb="FF7030A0"/>
+        <color rgb="FFD1621B"/>
       </right>
       <top style="medium">
-        <color rgb="FF7030A0"/>
+        <color rgb="FFD1621B"/>
       </top>
       <bottom style="medium">
-        <color rgb="FF7030A0"/>
+        <color rgb="FFD1621B"/>
       </bottom>
       <diagonal/>
     </border>
@@ -392,116 +401,124 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -525,7 +542,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FF00A651"/>
         </patternFill>
       </fill>
     </dxf>
@@ -535,11 +552,11 @@
         <charset val="1"/>
         <family val="0"/>
         <b val="1"/>
-        <color rgb="FF000000"/>
+        <color rgb="FF1A1A1A"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FF92D050"/>
+          <bgColor rgb="FF8CC63F"/>
         </patternFill>
       </fill>
     </dxf>
@@ -549,11 +566,11 @@
         <charset val="1"/>
         <family val="0"/>
         <b val="1"/>
-        <color rgb="FF000000"/>
+        <color rgb="FF1A1A1A"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFD966"/>
+          <bgColor rgb="FFFFD54F"/>
         </patternFill>
       </fill>
     </dxf>
@@ -563,11 +580,11 @@
         <charset val="1"/>
         <family val="0"/>
         <b val="1"/>
-        <color rgb="FF000000"/>
+        <color rgb="FF1A1A1A"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFF4B183"/>
+          <bgColor rgb="FFF4A261"/>
         </patternFill>
       </fill>
     </dxf>
@@ -581,7 +598,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF5050"/>
+          <bgColor rgb="FFE63946"/>
         </patternFill>
       </fill>
     </dxf>
@@ -599,17 +616,17 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF548235"/>
+      <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFBFBFBF"/>
+      <rgbColor rgb="FF0B7A75"/>
+      <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF878787"/>
-      <rgbColor rgb="FF8FAADC"/>
-      <rgbColor rgb="FF7030A0"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFDDEBF7"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF8E2C7D"/>
+      <rgbColor rgb="FFF3F5F9"/>
+      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FFF4A261"/>
       <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
@@ -623,27 +640,27 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FFA9D18E"/>
-      <rgbColor rgb="FFF4B183"/>
-      <rgbColor rgb="FFC9A3E0"/>
-      <rgbColor rgb="FFFFD966"/>
-      <rgbColor rgb="FF2E75B6"/>
+      <rgbColor rgb="FFFFE699"/>
+      <rgbColor rgb="FF7FC8C3"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFD3A0C8"/>
+      <rgbColor rgb="FFF2B27F"/>
+      <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF92D050"/>
-      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FF8CC63F"/>
+      <rgbColor rgb="FFFFD54F"/>
       <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF5050"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FFD1621B"/>
+      <rgbColor rgb="FF4F6D9A"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF1F3864"/>
-      <rgbColor rgb="FF00B050"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF00A651"/>
       <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FFC55A11"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="FF1A1A1A"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFE63946"/>
+      <rgbColor rgb="FF3D5A80"/>
+      <rgbColor rgb="FF14213D"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -675,7 +692,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>الصف كاملًا</a:t>
+              <a:t>الصف كاملًا  Whole Class</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -699,22 +716,22 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التحصيل"</c:f>
+              <c:f>"التحصيل Attainment"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التحصيل</c:v>
+                  <c:v>التحصيل Attainment</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="1f3864"/>
+              <a:srgbClr val="14213d"/>
             </a:solidFill>
             <a:ln w="0">
               <a:solidFill>
-                <a:srgbClr val="1f3864"/>
+                <a:srgbClr val="14213d"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -750,7 +767,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$7:$D$7</c:f>
+              <c:f>Dashboard!$H$7:$I$7</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -768,7 +785,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$8:$D$8</c:f>
+              <c:f>Dashboard!$H$8:$I$8</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
@@ -787,22 +804,22 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التقدم"</c:f>
+              <c:f>"التقدم Progress"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التقدم</c:v>
+                  <c:v>التقدم Progress</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="8faadc"/>
+              <a:srgbClr val="4f6d9a"/>
             </a:solidFill>
             <a:ln w="0">
               <a:solidFill>
-                <a:srgbClr val="8faadc"/>
+                <a:srgbClr val="4f6d9a"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -838,7 +855,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$7:$D$7</c:f>
+              <c:f>Dashboard!$H$7:$I$7</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -856,7 +873,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$9:$D$9</c:f>
+              <c:f>Dashboard!$H$9:$I$9</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
@@ -870,13 +887,13 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:gapWidth val="60"/>
-        <c:overlap val="0"/>
-        <c:axId val="81562439"/>
-        <c:axId val="27731922"/>
+        <c:gapWidth val="70"/>
+        <c:overlap val="-5"/>
+        <c:axId val="86844499"/>
+        <c:axId val="463674"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="81562439"/>
+        <c:axId val="86844499"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -908,7 +925,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27731922"/>
+        <c:crossAx val="463674"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -916,7 +933,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="27731922"/>
+        <c:axId val="463674"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -924,6 +941,16 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
         <c:numFmt formatCode="0%" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -950,9 +977,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81562439"/>
+        <c:crossAx val="86844499"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="0.25"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -1028,7 +1056,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>الإماراتيون</a:t>
+              <a:t>الإماراتيون  Emiratis</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1052,22 +1080,22 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التحصيل"</c:f>
+              <c:f>"التحصيل Attainment"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التحصيل</c:v>
+                  <c:v>التحصيل Attainment</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="548235"/>
+              <a:srgbClr val="0b7a75"/>
             </a:solidFill>
             <a:ln w="0">
               <a:solidFill>
-                <a:srgbClr val="548235"/>
+                <a:srgbClr val="0b7a75"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -1103,7 +1131,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$15:$D$15</c:f>
+              <c:f>Dashboard!$C$7:$D$7</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -1121,7 +1149,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$16:$D$16</c:f>
+              <c:f>Dashboard!$C$8:$D$8</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1140,22 +1168,22 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التقدم"</c:f>
+              <c:f>"التقدم Progress"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التقدم</c:v>
+                  <c:v>التقدم Progress</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="a9d18e"/>
+              <a:srgbClr val="7fc8c3"/>
             </a:solidFill>
             <a:ln w="0">
               <a:solidFill>
-                <a:srgbClr val="a9d18e"/>
+                <a:srgbClr val="7fc8c3"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -1191,7 +1219,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$15:$D$15</c:f>
+              <c:f>Dashboard!$C$7:$D$7</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -1209,7 +1237,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$17:$D$17</c:f>
+              <c:f>Dashboard!$C$9:$D$9</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1223,13 +1251,13 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:gapWidth val="60"/>
-        <c:overlap val="0"/>
-        <c:axId val="5298332"/>
-        <c:axId val="12279837"/>
+        <c:gapWidth val="70"/>
+        <c:overlap val="-5"/>
+        <c:axId val="52027838"/>
+        <c:axId val="68267142"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="5298332"/>
+        <c:axId val="52027838"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1261,7 +1289,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12279837"/>
+        <c:crossAx val="68267142"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1269,7 +1297,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="12279837"/>
+        <c:axId val="68267142"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1277,6 +1305,16 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
         <c:numFmt formatCode="0%" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1303,9 +1341,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5298332"/>
+        <c:crossAx val="52027838"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="0.25"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -1405,22 +1444,22 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التحصيل"</c:f>
+              <c:f>"التحصيل Attainment"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التحصيل</c:v>
+                  <c:v>التحصيل Attainment</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="c55a11"/>
+              <a:srgbClr val="d1621b"/>
             </a:solidFill>
             <a:ln w="0">
               <a:solidFill>
-                <a:srgbClr val="c55a11"/>
+                <a:srgbClr val="d1621b"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -1456,7 +1495,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$23:$D$23</c:f>
+              <c:f>Dashboard!$H$13:$I$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -1474,7 +1513,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$24:$D$24</c:f>
+              <c:f>Dashboard!$H$14:$I$14</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1493,22 +1532,22 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التقدم"</c:f>
+              <c:f>"التقدم Progress"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التقدم</c:v>
+                  <c:v>التقدم Progress</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="f4b183"/>
+              <a:srgbClr val="f2b27f"/>
             </a:solidFill>
             <a:ln w="0">
               <a:solidFill>
-                <a:srgbClr val="f4b183"/>
+                <a:srgbClr val="f2b27f"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -1544,7 +1583,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$23:$D$23</c:f>
+              <c:f>Dashboard!$H$13:$I$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -1562,7 +1601,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$25:$D$25</c:f>
+              <c:f>Dashboard!$H$15:$I$15</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1576,13 +1615,13 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:gapWidth val="60"/>
-        <c:overlap val="0"/>
-        <c:axId val="61430187"/>
-        <c:axId val="43799199"/>
+        <c:gapWidth val="70"/>
+        <c:overlap val="-5"/>
+        <c:axId val="67581601"/>
+        <c:axId val="83338174"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="61430187"/>
+        <c:axId val="67581601"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1614,7 +1653,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43799199"/>
+        <c:crossAx val="83338174"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1622,7 +1661,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="43799199"/>
+        <c:axId val="83338174"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1630,6 +1669,16 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
         <c:numFmt formatCode="0%" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1656,9 +1705,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61430187"/>
+        <c:crossAx val="67581601"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="0.25"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -1758,22 +1808,22 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التحصيل"</c:f>
+              <c:f>"التحصيل Attainment"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التحصيل</c:v>
+                  <c:v>التحصيل Attainment</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="7030a0"/>
+              <a:srgbClr val="8e2c7d"/>
             </a:solidFill>
             <a:ln w="0">
               <a:solidFill>
-                <a:srgbClr val="7030a0"/>
+                <a:srgbClr val="8e2c7d"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -1809,7 +1859,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$31:$D$31</c:f>
+              <c:f>Dashboard!$C$13:$D$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -1827,7 +1877,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$32:$D$32</c:f>
+              <c:f>Dashboard!$C$14:$D$14</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1846,22 +1896,22 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>"التقدم"</c:f>
+              <c:f>"التقدم Progress"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>التقدم</c:v>
+                  <c:v>التقدم Progress</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="c9a3e0"/>
+              <a:srgbClr val="d3a0c8"/>
             </a:solidFill>
             <a:ln w="0">
               <a:solidFill>
-                <a:srgbClr val="c9a3e0"/>
+                <a:srgbClr val="d3a0c8"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -1897,7 +1947,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Dashboard!$C$31:$D$31</c:f>
+              <c:f>Dashboard!$C$13:$D$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="1"/>
                 <c:lvl>
@@ -1915,7 +1965,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$33:$D$33</c:f>
+              <c:f>Dashboard!$C$15:$D$15</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1929,13 +1979,13 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:gapWidth val="60"/>
-        <c:overlap val="0"/>
-        <c:axId val="75508505"/>
-        <c:axId val="82428111"/>
+        <c:gapWidth val="70"/>
+        <c:overlap val="-5"/>
+        <c:axId val="2695673"/>
+        <c:axId val="40580294"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="75508505"/>
+        <c:axId val="2695673"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1967,7 +2017,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82428111"/>
+        <c:crossAx val="40580294"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1975,7 +2025,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="82428111"/>
+        <c:axId val="40580294"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1983,6 +2033,16 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
         <c:numFmt formatCode="0%" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -2009,9 +2069,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75508505"/>
+        <c:crossAx val="2695673"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="0.25"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -2066,15 +2127,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>-39240</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>156960</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1158480</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>187200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2082,8 +2143,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-10170000" y="1562040"/>
-        <a:ext cx="4319640" cy="1871640"/>
+        <a:off x="5427360" y="5667480"/>
+        <a:ext cx="4823640" cy="2663640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2095,16 +2156,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>-39240</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>156960</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1158480</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>187200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2112,8 +2173,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-10170000" y="3657600"/>
-        <a:ext cx="4319640" cy="1871640"/>
+        <a:off x="141120" y="5667480"/>
+        <a:ext cx="4823640" cy="2663640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2126,15 +2187,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>-39240</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>157320</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1158480</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>187200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2142,8 +2203,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-10170000" y="5753160"/>
-        <a:ext cx="4319640" cy="1871640"/>
+        <a:off x="5427360" y="8524800"/>
+        <a:ext cx="4823640" cy="2663640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2155,16 +2216,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>-39240</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>157320</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1158480</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>187200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2172,8 +2233,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-10170000" y="7848720"/>
-        <a:ext cx="4319640" cy="1871640"/>
+        <a:off x="141120" y="8524800"/>
+        <a:ext cx="4823640" cy="2663640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2366,267 +2427,924 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E33"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1" t="s">
+    <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1"/>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1"/>
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="2" t="s">
+      <c r="F2" s="1"/>
+      <c r="G2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1"/>
+      <c r="B3" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="2" t="s">
+      <c r="E3" s="4"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="1"/>
+    </row>
+    <row r="4" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1"/>
+      <c r="B6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="8" t="n">
+        <f aca="false">B3</f>
         <v>28</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="5" t="n">
-        <f aca="false">C4</f>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="6"/>
-      <c r="C7" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="K6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="D7" s="9" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="7" t="s">
+      <c r="E7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="F7" s="1"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="K7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1"/>
+      <c r="B8" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="1"/>
+      <c r="G8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="15" t="n">
         <v>0.8</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="I8" s="15" t="n">
         <v>0.35</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="J8" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="K8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+      <c r="B9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="1"/>
+      <c r="G9" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I9" s="15" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J9" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="K9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+    </row>
+    <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+      <c r="B12" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="1"/>
+      <c r="G12" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="K12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="1"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="I13" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="J13" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="K13" s="1"/>
+    </row>
+    <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1"/>
+      <c r="B14" s="23" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="7" t="s">
+      <c r="C14" s="24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E14" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I14" s="27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J14" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="K14" s="1"/>
+    </row>
+    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1"/>
+      <c r="B15" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="24" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E15" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="27" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J15" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="8" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D9" s="8" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="11" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="12"/>
-      <c r="C15" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D16" s="14" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="14" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D17" s="14" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E17" s="15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="17" t="n">
-        <v>4</v>
-      </c>
+      <c r="K15" s="1"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+    </row>
+    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1"/>
+      <c r="B19" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
+      <c r="J19" s="29"/>
+      <c r="K19" s="1"/>
+    </row>
+    <row r="20" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="18"/>
-      <c r="C23" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="C24" s="20" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D24" s="20" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C25" s="20" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D25" s="20" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E25" s="21" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="23" t="n">
-        <v>3</v>
-      </c>
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="24"/>
-      <c r="C31" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="E31" s="24" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="C32" s="26" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="D32" s="26" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E32" s="27" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="C33" s="26" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="D33" s="26" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="E33" s="27" t="s">
-        <v>18</v>
-      </c>
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+      <c r="J38" s="1"/>
+      <c r="K38" s="1"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1"/>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="J40" s="1"/>
+      <c r="K40" s="1"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+      <c r="I41" s="1"/>
+      <c r="J41" s="1"/>
+      <c r="K41" s="1"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="1"/>
+      <c r="D42" s="1"/>
+      <c r="E42" s="1"/>
+      <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+      <c r="I42" s="1"/>
+      <c r="J42" s="1"/>
+      <c r="K42" s="1"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1"/>
+      <c r="B43" s="1"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+      <c r="E43" s="1"/>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1"/>
+      <c r="I43" s="1"/>
+      <c r="J43" s="1"/>
+      <c r="K43" s="1"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1"/>
+      <c r="B44" s="1"/>
+      <c r="C44" s="1"/>
+      <c r="D44" s="1"/>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+      <c r="I44" s="1"/>
+      <c r="J44" s="1"/>
+      <c r="K44" s="1"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1"/>
+      <c r="B45" s="1"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="1"/>
+      <c r="E45" s="1"/>
+      <c r="F45" s="1"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
+      <c r="I45" s="1"/>
+      <c r="J45" s="1"/>
+      <c r="K45" s="1"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1"/>
+      <c r="B46" s="1"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="1"/>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+      <c r="I46" s="1"/>
+      <c r="J46" s="1"/>
+      <c r="K46" s="1"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1"/>
+      <c r="B47" s="1"/>
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+      <c r="I47" s="1"/>
+      <c r="J47" s="1"/>
+      <c r="K47" s="1"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1"/>
+      <c r="B48" s="1"/>
+      <c r="C48" s="1"/>
+      <c r="D48" s="1"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+      <c r="I48" s="1"/>
+      <c r="J48" s="1"/>
+      <c r="K48" s="1"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1"/>
+      <c r="B49" s="1"/>
+      <c r="C49" s="1"/>
+      <c r="D49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+      <c r="I49" s="1"/>
+      <c r="J49" s="1"/>
+      <c r="K49" s="1"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="1"/>
+      <c r="B50" s="1"/>
+      <c r="C50" s="1"/>
+      <c r="D50" s="1"/>
+      <c r="E50" s="1"/>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+      <c r="I50" s="1"/>
+      <c r="J50" s="1"/>
+      <c r="K50" s="1"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1"/>
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+      <c r="D51" s="1"/>
+      <c r="E51" s="1"/>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1"/>
+      <c r="I51" s="1"/>
+      <c r="J51" s="1"/>
+      <c r="K51" s="1"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1"/>
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1"/>
+      <c r="J52" s="1"/>
+      <c r="K52" s="1"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1"/>
+      <c r="B53" s="1"/>
+      <c r="C53" s="1"/>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+      <c r="I53" s="1"/>
+      <c r="J53" s="1"/>
+      <c r="K53" s="1"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="1"/>
+      <c r="B54" s="1"/>
+      <c r="C54" s="1"/>
+      <c r="D54" s="1"/>
+      <c r="E54" s="1"/>
+      <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+      <c r="I54" s="1"/>
+      <c r="J54" s="1"/>
+      <c r="K54" s="1"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1"/>
+      <c r="B55" s="1"/>
+      <c r="C55" s="1"/>
+      <c r="D55" s="1"/>
+      <c r="E55" s="1"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
+      <c r="I55" s="1"/>
+      <c r="J55" s="1"/>
+      <c r="K55" s="1"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1"/>
+      <c r="B56" s="1"/>
+      <c r="C56" s="1"/>
+      <c r="D56" s="1"/>
+      <c r="E56" s="1"/>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+      <c r="I56" s="1"/>
+      <c r="J56" s="1"/>
+      <c r="K56" s="1"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1"/>
+      <c r="B57" s="1"/>
+      <c r="C57" s="1"/>
+      <c r="D57" s="1"/>
+      <c r="E57" s="1"/>
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
+      <c r="I57" s="1"/>
+      <c r="J57" s="1"/>
+      <c r="K57" s="1"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1"/>
+      <c r="B58" s="1"/>
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+      <c r="I58" s="1"/>
+      <c r="J58" s="1"/>
+      <c r="K58" s="1"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1"/>
+      <c r="B59" s="1"/>
+      <c r="C59" s="1"/>
+      <c r="D59" s="1"/>
+      <c r="E59" s="1"/>
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1"/>
+      <c r="I59" s="1"/>
+      <c r="J59" s="1"/>
+      <c r="K59" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="C4:E4"/>
+  <mergeCells count="12">
+    <mergeCell ref="B1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="G2:J2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="G3:J3"/>
     <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="B19:J19"/>
   </mergeCells>
-  <conditionalFormatting sqref="E8:E40">
+  <conditionalFormatting sqref="E8:E9">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>E8="Outstanding"</formula>
     </cfRule>
@@ -2643,19 +3361,74 @@
       <formula>E8="Weak"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E8:E9 E16:E17 E24:E25 E32:E33" type="list">
+  <conditionalFormatting sqref="J8:J9">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>J8="Outstanding"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>J8="Very Good"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>J8="Good"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>J8="Acceptable"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+      <formula>J8="Weak"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E14:E15">
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>E14="Outstanding"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>E14="Very Good"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>E14="Good"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>E14="Acceptable"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+      <formula>E14="Weak"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J14:J15">
+    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>J14="Outstanding"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>J14="Very Good"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>J14="Good"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>J14="Acceptable"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+      <formula>J14="Weak"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E8:E9 J8:J9 E14:E15 J14:J15" type="list">
       <formula1>"Outstanding,Very Good,Good,Acceptable,Weak"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" error="أدخل نسبة بين 0% و100%" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C8:D9 C16:D17 C24:D25 C32:D33" type="decimal">
+    <dataValidation allowBlank="false" error="أدخل نسبة بين 0% و100%" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C8:D9 H8:I9 C14:D15 H14:I15" type="decimal">
       <formula1>0</formula1>
       <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="أدخل رقمًا صحيحًا" errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E6 E12 J12" type="whole">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>